<commit_message>
modifico usuario pruebas y adicional Amy
</commit_message>
<xml_diff>
--- a/backend/data/tecnicos.xlsx
+++ b/backend/data/tecnicos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WILMAR\Diagnostico03\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6580EB8C-958D-4FED-BB97-209351028BFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8B5F49E-CE8D-4222-89ED-478BA9955305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="65">
   <si>
     <t>Cédula</t>
   </si>
@@ -202,13 +202,19 @@
     <t>Wilmar Eulises Franco Beltran</t>
   </si>
   <si>
-    <t>Pruebas26.</t>
-  </si>
-  <si>
     <t>Pruebas Probando</t>
   </si>
   <si>
     <t>Probador experto</t>
+  </si>
+  <si>
+    <t>Bb010416</t>
+  </si>
+  <si>
+    <t>Amy Franco</t>
+  </si>
+  <si>
+    <t>Pruebas26*</t>
   </si>
 </sst>
 </file>
@@ -585,10 +591,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="30.25" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -605,7 +614,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -622,7 +631,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>88160957</v>
       </c>
@@ -639,7 +648,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>80845492</v>
       </c>
@@ -656,7 +665,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1033820304</v>
       </c>
@@ -673,7 +682,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1000734283</v>
       </c>
@@ -690,7 +699,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>79133058</v>
       </c>
@@ -707,7 +716,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>11590324</v>
       </c>
@@ -724,7 +733,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>80140585</v>
       </c>
@@ -741,7 +750,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>80063906</v>
       </c>
@@ -758,7 +767,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1010204069</v>
       </c>
@@ -775,7 +784,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1233900389</v>
       </c>
@@ -792,7 +801,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1033721088</v>
       </c>
@@ -809,7 +818,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10301508</v>
       </c>
@@ -826,7 +835,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>80796479</v>
       </c>
@@ -843,7 +852,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1020760934</v>
       </c>
@@ -860,7 +869,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1062304838</v>
       </c>
@@ -877,7 +886,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>40437175</v>
       </c>
@@ -894,7 +903,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1076624363</v>
       </c>
@@ -911,7 +920,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1023932651</v>
       </c>
@@ -928,7 +937,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>80240931</v>
       </c>
@@ -945,7 +954,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1030667140</v>
       </c>
@@ -962,7 +971,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1031131751</v>
       </c>
@@ -979,7 +988,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1116544966</v>
       </c>
@@ -996,7 +1005,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1022338458</v>
       </c>
@@ -1013,7 +1022,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>80056982</v>
       </c>
@@ -1030,7 +1039,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1121855145</v>
       </c>
@@ -1052,16 +1061,33 @@
         <v>123456789</v>
       </c>
       <c r="B28" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" t="s">
         <v>60</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>61</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>1122931979</v>
+      </c>
+      <c r="B29" t="s">
         <v>62</v>
       </c>
-      <c r="E28" t="s">
-        <v>16</v>
+      <c r="C29" t="s">
+        <v>63</v>
+      </c>
+      <c r="D29" t="s">
+        <v>6</v>
+      </c>
+      <c r="E29" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>